<commit_message>
compleate Tests adn excel file
</commit_message>
<xml_diff>
--- a/Report/Res.xlsx
+++ b/Report/Res.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Amir\Uni\Course\Master\RT2\Assignments\03\Amirmat\Research_Track1_Assignment1\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8534D506-5A62-48F1-95F9-1843929F52DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF046CDE-4F6D-4DB7-AB75-55B76BC95269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Test Number</t>
   </si>
@@ -64,16 +64,20 @@
   <si>
     <t>t</t>
   </si>
+  <si>
+    <t>P-value</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.00000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
+    <numFmt numFmtId="179" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,16 +85,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -98,22 +114,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -392,672 +435,983 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E50"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
-        <v>3</v>
-      </c>
-      <c r="E2" s="1"/>
+      <c r="B2" s="2">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>38.393619999999999</v>
+      </c>
+      <c r="D2" s="2">
+        <v>48.369840000000003</v>
+      </c>
+      <c r="E2" s="2">
+        <f xml:space="preserve"> D2 - C2</f>
+        <v>9.976220000000005</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <f xml:space="preserve"> A2+1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>39.113669999999999</v>
+      </c>
+      <c r="D3" s="2">
+        <v>49.659750000000003</v>
+      </c>
+      <c r="E3" s="2">
+        <f t="shared" ref="E3:E46" si="0" xml:space="preserve"> D3 - C3</f>
+        <v>10.546080000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <f t="shared" ref="A4:A46" si="1" xml:space="preserve"> A3+1</f>
         <v>3</v>
       </c>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <f t="shared" ref="A4:A46" si="0" xml:space="preserve"> A3+1</f>
-        <v>3</v>
-      </c>
-      <c r="B4" s="4">
-        <v>3</v>
-      </c>
-      <c r="E4" s="1"/>
+      <c r="B4" s="2">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>38.53369</v>
+      </c>
+      <c r="D4" s="2">
+        <v>49.326979999999999</v>
+      </c>
+      <c r="E4" s="2">
+        <f t="shared" si="0"/>
+        <v>10.793289999999999</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="B5" s="4">
-        <v>3</v>
-      </c>
-      <c r="E5" s="1"/>
+      <c r="A5" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2">
+        <v>37.206249999999997</v>
+      </c>
+      <c r="D5" s="2">
+        <v>50.145690000000002</v>
+      </c>
+      <c r="E5" s="2">
+        <f t="shared" si="0"/>
+        <v>12.939440000000005</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <f t="shared" si="0"/>
+      <c r="A6" s="2">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B6" s="4">
-        <v>3</v>
-      </c>
-      <c r="E6" s="1"/>
+      <c r="B6" s="2">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2">
+        <v>38.914580000000001</v>
+      </c>
+      <c r="D6" s="2">
+        <v>49.786529999999999</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" si="0"/>
+        <v>10.871949999999998</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="B7" s="4">
-        <v>3</v>
-      </c>
-      <c r="E7" s="1"/>
+      <c r="A7" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2">
+        <v>38.014589999999998</v>
+      </c>
+      <c r="D7" s="2">
+        <v>50.964869999999998</v>
+      </c>
+      <c r="E7" s="2">
+        <f t="shared" si="0"/>
+        <v>12.950279999999999</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <f t="shared" si="0"/>
+      <c r="A8" s="2">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="B8" s="4">
-        <v>3</v>
-      </c>
-      <c r="E8" s="1"/>
+      <c r="B8" s="2">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2">
+        <v>39.254779999999997</v>
+      </c>
+      <c r="D8" s="2">
+        <v>52.469749999999998</v>
+      </c>
+      <c r="E8" s="2">
+        <f t="shared" si="0"/>
+        <v>13.214970000000001</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="B9" s="4">
-        <v>3</v>
-      </c>
-      <c r="E9" s="1"/>
+      <c r="A9" s="2">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2">
+        <v>38.658790000000003</v>
+      </c>
+      <c r="D9" s="2">
+        <v>51.456980000000001</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="0"/>
+        <v>12.798189999999998</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <f t="shared" si="0"/>
+      <c r="A10" s="2">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="B10" s="4">
-        <v>3</v>
-      </c>
-      <c r="E10" s="1"/>
+      <c r="B10" s="2">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2">
+        <v>40.749859999999998</v>
+      </c>
+      <c r="D10" s="2">
+        <v>51.24689</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>10.497030000000002</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <f t="shared" si="0"/>
+      <c r="A11" s="2">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="B11" s="4">
-        <v>3</v>
-      </c>
-      <c r="E11" s="1"/>
+      <c r="B11" s="2">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>39.789630000000002</v>
+      </c>
+      <c r="D11" s="2">
+        <v>50.79354</v>
+      </c>
+      <c r="E11" s="2">
+        <f t="shared" si="0"/>
+        <v>11.003909999999998</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <f t="shared" si="0"/>
+      <c r="A12" s="2">
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="B12" s="4">
-        <v>3</v>
-      </c>
-      <c r="E12" s="1"/>
+      <c r="B12" s="2">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2">
+        <v>40.35689</v>
+      </c>
+      <c r="D12" s="2">
+        <v>53.236980000000003</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="0"/>
+        <v>12.880090000000003</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <f t="shared" si="0"/>
+      <c r="A13" s="2">
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="B13" s="4">
-        <v>3</v>
-      </c>
-      <c r="E13" s="1"/>
+      <c r="B13" s="2">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2">
+        <v>38.968470000000003</v>
+      </c>
+      <c r="D13" s="2">
+        <v>52.34975</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="0"/>
+        <v>13.381279999999997</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <f t="shared" si="0"/>
+      <c r="A14" s="2">
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="B14" s="4">
-        <v>3</v>
-      </c>
-      <c r="E14" s="1"/>
+      <c r="B14" s="2">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2">
+        <v>38.014650000000003</v>
+      </c>
+      <c r="D14" s="2">
+        <v>52.654389999999999</v>
+      </c>
+      <c r="E14" s="2">
+        <f t="shared" si="0"/>
+        <v>14.639739999999996</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <f t="shared" si="0"/>
+      <c r="A15" s="2">
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="B15" s="4">
-        <v>3</v>
-      </c>
-      <c r="E15" s="1"/>
+      <c r="B15" s="2">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2">
+        <v>39.115690000000001</v>
+      </c>
+      <c r="D15" s="2">
+        <v>53.011539999999997</v>
+      </c>
+      <c r="E15" s="2">
+        <f t="shared" si="0"/>
+        <v>13.895849999999996</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <f t="shared" si="0"/>
+      <c r="A16" s="2">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="B16" s="4">
-        <v>3</v>
-      </c>
-      <c r="E16" s="1"/>
+      <c r="B16" s="2">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2">
+        <v>39.789639999999999</v>
+      </c>
+      <c r="D16" s="2">
+        <v>53.24615</v>
+      </c>
+      <c r="E16" s="2">
+        <f t="shared" si="0"/>
+        <v>13.456510000000002</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <f t="shared" si="0"/>
+      <c r="A17" s="2">
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="B17" s="1">
-        <v>6</v>
-      </c>
-      <c r="C17" s="2">
+      <c r="B17" s="2">
+        <v>6</v>
+      </c>
+      <c r="C17" s="3">
         <v>54.959874868392902</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="4">
         <v>84.652799999999999</v>
       </c>
-      <c r="E17" s="1"/>
+      <c r="E17" s="2">
+        <f t="shared" si="0"/>
+        <v>29.692925131607097</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <f t="shared" si="0"/>
+      <c r="A18" s="2">
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="B18" s="1">
-        <v>6</v>
-      </c>
-      <c r="C18" s="2">
+      <c r="B18" s="2">
+        <v>6</v>
+      </c>
+      <c r="C18" s="3">
         <v>55.274461746215799</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>85.44914</v>
       </c>
-      <c r="E18" s="1"/>
+      <c r="E18" s="2">
+        <f t="shared" si="0"/>
+        <v>30.174678253784201</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <f t="shared" si="0"/>
+      <c r="A19" s="2">
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="B19" s="1">
-        <v>6</v>
-      </c>
-      <c r="C19" s="2">
+      <c r="B19" s="2">
+        <v>6</v>
+      </c>
+      <c r="C19" s="3">
         <v>52.361139774322503</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="2">
         <v>84.469549999999998</v>
       </c>
-      <c r="E19" s="1"/>
+      <c r="E19" s="2">
+        <f t="shared" si="0"/>
+        <v>32.108410225677495</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <f t="shared" si="0"/>
+      <c r="A20" s="2">
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="B20" s="1">
-        <v>6</v>
-      </c>
-      <c r="C20" s="2">
+      <c r="B20" s="2">
+        <v>6</v>
+      </c>
+      <c r="C20" s="3">
         <v>54.494693517684901</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <v>85.056229999999999</v>
       </c>
-      <c r="E20" s="1"/>
+      <c r="E20" s="2">
+        <f t="shared" si="0"/>
+        <v>30.561536482315098</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <f t="shared" si="0"/>
+      <c r="A21" s="2">
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="B21" s="1">
-        <v>6</v>
-      </c>
-      <c r="C21" s="2">
+      <c r="B21" s="2">
+        <v>6</v>
+      </c>
+      <c r="C21" s="3">
         <v>53.376106500625603</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="2">
         <v>85.262860000000003</v>
       </c>
-      <c r="E21" s="1"/>
+      <c r="E21" s="2">
+        <f t="shared" si="0"/>
+        <v>31.8867534993744</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <f t="shared" si="0"/>
+      <c r="A22" s="2">
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="B22" s="1">
-        <v>6</v>
-      </c>
-      <c r="C22" s="2">
+      <c r="B22" s="2">
+        <v>6</v>
+      </c>
+      <c r="C22" s="3">
         <v>54.613642930984497</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="2">
         <v>85.144090000000006</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="E22" s="2">
+        <f t="shared" si="0"/>
+        <v>30.530447069015509</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <f t="shared" si="0"/>
+      <c r="A23" s="2">
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="B23" s="1">
-        <v>6</v>
-      </c>
-      <c r="C23" s="2">
+      <c r="B23" s="2">
+        <v>6</v>
+      </c>
+      <c r="C23" s="3">
         <v>58.057340383529599</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="2">
         <v>84.786169999999998</v>
       </c>
-      <c r="E23" s="1"/>
+      <c r="E23" s="2">
+        <f t="shared" si="0"/>
+        <v>26.728829616470399</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <f t="shared" si="0"/>
+      <c r="A24" s="2">
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="B24" s="1">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2">
+      <c r="B24" s="2">
+        <v>6</v>
+      </c>
+      <c r="C24" s="3">
         <v>59.334924936294499</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="2">
         <v>84.369529999999997</v>
       </c>
-      <c r="E24" s="1"/>
+      <c r="E24" s="2">
+        <f t="shared" si="0"/>
+        <v>25.034605063705499</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <f t="shared" si="0"/>
+      <c r="A25" s="2">
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="B25" s="1">
-        <v>6</v>
-      </c>
-      <c r="C25" s="2">
+      <c r="B25" s="2">
+        <v>6</v>
+      </c>
+      <c r="C25" s="3">
         <v>55.130685567855799</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="2">
         <v>85.046859999999995</v>
       </c>
-      <c r="E25" s="1"/>
+      <c r="E25" s="2">
+        <f t="shared" si="0"/>
+        <v>29.916174432144196</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <f t="shared" si="0"/>
+      <c r="A26" s="2">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="B26" s="1">
-        <v>6</v>
-      </c>
-      <c r="C26" s="2">
+      <c r="B26" s="2">
+        <v>6</v>
+      </c>
+      <c r="C26" s="3">
         <v>59.192314386367798</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="2">
         <v>84.77364</v>
       </c>
-      <c r="E26" s="1"/>
+      <c r="E26" s="2">
+        <f t="shared" si="0"/>
+        <v>25.581325613632202</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <f t="shared" si="0"/>
+      <c r="A27" s="2">
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="B27" s="1">
-        <v>6</v>
-      </c>
-      <c r="C27" s="2">
+      <c r="B27" s="2">
+        <v>6</v>
+      </c>
+      <c r="C27" s="3">
         <v>55.940476894378598</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="2">
         <v>84.877070000000003</v>
       </c>
-      <c r="E27" s="1"/>
+      <c r="E27" s="2">
+        <f t="shared" si="0"/>
+        <v>28.936593105621405</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <f t="shared" si="0"/>
+      <c r="A28" s="2">
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="B28" s="1">
-        <v>6</v>
-      </c>
-      <c r="C28" s="2">
+      <c r="B28" s="2">
+        <v>6</v>
+      </c>
+      <c r="C28" s="3">
         <v>55.067856788635197</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="2">
         <v>84.82687</v>
       </c>
-      <c r="E28" s="1"/>
+      <c r="E28" s="2">
+        <f t="shared" si="0"/>
+        <v>29.759013211364802</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <f t="shared" si="0"/>
+      <c r="A29" s="2">
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="B29" s="1">
-        <v>6</v>
-      </c>
-      <c r="C29" s="2">
+      <c r="B29" s="2">
+        <v>6</v>
+      </c>
+      <c r="C29" s="3">
         <v>54.453131914138702</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="2">
         <v>84.478229999999996</v>
       </c>
-      <c r="E29" s="1"/>
+      <c r="E29" s="2">
+        <f t="shared" si="0"/>
+        <v>30.025098085861295</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <f t="shared" si="0"/>
+      <c r="A30" s="2">
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="B30" s="1">
-        <v>6</v>
-      </c>
-      <c r="C30" s="2">
+      <c r="B30" s="2">
+        <v>6</v>
+      </c>
+      <c r="C30" s="3">
         <v>55.049853324890101</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="2">
         <v>84.074349999999995</v>
       </c>
-      <c r="E30" s="1"/>
+      <c r="E30" s="2">
+        <f t="shared" si="0"/>
+        <v>29.024496675109894</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <f t="shared" si="0"/>
+      <c r="A31" s="2">
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="B31" s="1">
-        <v>6</v>
-      </c>
-      <c r="C31" s="2">
+      <c r="B31" s="2">
+        <v>6</v>
+      </c>
+      <c r="C31" s="3">
         <v>54.397413253784102</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="4">
         <v>84.998500000000007</v>
       </c>
-      <c r="E31" s="1"/>
+      <c r="E31" s="2">
+        <f t="shared" si="0"/>
+        <v>30.601086746215906</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
-        <f t="shared" si="0"/>
+      <c r="A32" s="2">
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="B32" s="1">
-        <v>8</v>
-      </c>
-      <c r="C32" s="2">
+      <c r="B32" s="2">
+        <v>8</v>
+      </c>
+      <c r="C32" s="3">
         <v>78.262053728103595</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="2">
         <v>116.657028</v>
       </c>
-      <c r="E32" s="1"/>
+      <c r="E32" s="2">
+        <f t="shared" si="0"/>
+        <v>38.394974271896402</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
-        <f t="shared" si="0"/>
+      <c r="A33" s="2">
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="B33" s="1">
-        <v>8</v>
-      </c>
-      <c r="C33" s="2">
+      <c r="B33" s="2">
+        <v>8</v>
+      </c>
+      <c r="C33" s="3">
         <v>75.808310508727999</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="2">
         <v>116.31923999999999</v>
       </c>
-      <c r="E33" s="1"/>
+      <c r="E33" s="2">
+        <f t="shared" si="0"/>
+        <v>40.510929491271995</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <f t="shared" si="0"/>
+      <c r="A34" s="2">
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
-      <c r="B34" s="1">
-        <v>8</v>
-      </c>
-      <c r="C34" s="2">
+      <c r="B34" s="2">
+        <v>8</v>
+      </c>
+      <c r="C34" s="3">
         <v>75.558684110641394</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="2">
         <v>116.99526</v>
       </c>
-      <c r="E34" s="1"/>
+      <c r="E34" s="2">
+        <f t="shared" si="0"/>
+        <v>41.436575889358608</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <f t="shared" si="0"/>
+      <c r="A35" s="2">
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="B35" s="1">
-        <v>8</v>
-      </c>
-      <c r="C35" s="2">
+      <c r="B35" s="2">
+        <v>8</v>
+      </c>
+      <c r="C35" s="3">
         <v>78.6530117988586</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="2">
         <v>116.06432</v>
       </c>
-      <c r="E35" s="1"/>
+      <c r="E35" s="2">
+        <f t="shared" si="0"/>
+        <v>37.411308201141395</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <f t="shared" si="0"/>
+      <c r="A36" s="2">
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="B36" s="1">
-        <v>8</v>
-      </c>
-      <c r="C36" s="2">
+      <c r="B36" s="2">
+        <v>8</v>
+      </c>
+      <c r="C36" s="3">
         <v>72.045760154724107</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="2">
         <v>118.91829</v>
       </c>
+      <c r="E36" s="2">
+        <f t="shared" si="0"/>
+        <v>46.872529845275892</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <f t="shared" si="0"/>
+      <c r="A37" s="2">
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="B37" s="1">
-        <v>8</v>
-      </c>
-      <c r="C37" s="2">
+      <c r="B37" s="2">
+        <v>8</v>
+      </c>
+      <c r="C37" s="3">
         <v>77.804898262023897</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="2">
         <v>115.75485</v>
       </c>
+      <c r="E37" s="2">
+        <f t="shared" si="0"/>
+        <v>37.949951737976107</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <f t="shared" si="0"/>
+      <c r="A38" s="2">
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="B38" s="1">
-        <v>8</v>
-      </c>
-      <c r="C38" s="2">
+      <c r="B38" s="2">
+        <v>8</v>
+      </c>
+      <c r="C38" s="3">
         <v>76.690699815750094</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="2">
         <v>116.05548</v>
       </c>
+      <c r="E38" s="2">
+        <f t="shared" si="0"/>
+        <v>39.364780184249909</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <f t="shared" si="0"/>
+      <c r="A39" s="2">
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="B39" s="1">
-        <v>8</v>
-      </c>
-      <c r="C39" s="2">
+      <c r="B39" s="2">
+        <v>8</v>
+      </c>
+      <c r="C39" s="3">
         <v>74.823342323303194</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="2">
         <v>114.75794999999999</v>
       </c>
+      <c r="E39" s="2">
+        <f t="shared" si="0"/>
+        <v>39.9346076766968</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <f t="shared" si="0"/>
+      <c r="A40" s="2">
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
-      <c r="B40" s="1">
-        <v>8</v>
-      </c>
-      <c r="C40" s="2">
+      <c r="B40" s="2">
+        <v>8</v>
+      </c>
+      <c r="C40" s="3">
         <v>74.272506237030001</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="2">
         <v>113.37381000000001</v>
       </c>
+      <c r="E40" s="2">
+        <f t="shared" si="0"/>
+        <v>39.101303762970005</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <f t="shared" si="0"/>
+      <c r="A41" s="2">
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="B41" s="1">
-        <v>8</v>
-      </c>
-      <c r="C41" s="2">
+      <c r="B41" s="2">
+        <v>8</v>
+      </c>
+      <c r="C41" s="3">
         <v>70.117750883102403</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="2">
         <v>116.49312</v>
       </c>
+      <c r="E41" s="2">
+        <f t="shared" si="0"/>
+        <v>46.375369116897602</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
-        <f t="shared" si="0"/>
+      <c r="A42" s="2">
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="B42" s="1">
-        <v>8</v>
-      </c>
-      <c r="C42" s="2">
+      <c r="B42" s="2">
+        <v>8</v>
+      </c>
+      <c r="C42" s="3">
         <v>74.899099588394094</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="2">
         <v>116.00306</v>
       </c>
+      <c r="E42" s="2">
+        <f t="shared" si="0"/>
+        <v>41.103960411605911</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <f t="shared" si="0"/>
+      <c r="A43" s="2">
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
-      <c r="B43" s="1">
-        <v>8</v>
-      </c>
-      <c r="C43" s="2">
+      <c r="B43" s="2">
+        <v>8</v>
+      </c>
+      <c r="C43" s="3">
         <v>76.601675033569293</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="2">
         <v>119.4113</v>
       </c>
+      <c r="E43" s="2">
+        <f t="shared" si="0"/>
+        <v>42.809624966430704</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
-        <f t="shared" si="0"/>
+      <c r="A44" s="2">
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
-      <c r="B44" s="1">
-        <v>8</v>
-      </c>
-      <c r="C44" s="2">
+      <c r="B44" s="2">
+        <v>8</v>
+      </c>
+      <c r="C44" s="3">
         <v>79.258589982986393</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="2">
         <v>116.68213</v>
       </c>
+      <c r="E44" s="2">
+        <f t="shared" si="0"/>
+        <v>37.423540017013607</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
-        <f t="shared" si="0"/>
+      <c r="A45" s="2">
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
-      <c r="B45" s="1">
-        <v>8</v>
-      </c>
-      <c r="C45" s="2">
+      <c r="B45" s="2">
+        <v>8</v>
+      </c>
+      <c r="C45" s="3">
         <v>79.327092885970998</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="2">
         <v>120.26223</v>
       </c>
+      <c r="E45" s="2">
+        <f t="shared" si="0"/>
+        <v>40.935137114029004</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
-        <f t="shared" si="0"/>
+      <c r="A46" s="2">
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="B46" s="1">
-        <v>8</v>
-      </c>
-      <c r="C46" s="2">
+      <c r="B46" s="2">
+        <v>8</v>
+      </c>
+      <c r="C46" s="3">
         <v>78.2503178119659</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="2">
         <v>116.50902000000001</v>
       </c>
+      <c r="E46" s="2">
+        <f t="shared" si="0"/>
+        <v>38.258702188034107</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5">
+        <f>AVERAGE(C2:C46)</f>
+        <v>56.865611331405631</v>
+      </c>
+      <c r="D47" s="5">
+        <f>AVERAGE(D2:D46)</f>
+        <v>84.249835733333342</v>
+      </c>
+      <c r="E47" s="5">
+        <f>AVERAGE(E2:E46)</f>
+        <v>27.384224401927714</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+      <c r="A48" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5">
+        <f>_xlfn.STDEV.S(C2:C46)</f>
+        <v>15.49971717006976</v>
+      </c>
+      <c r="D48" s="5">
+        <f>_xlfn.STDEV.S(D2:D46)</f>
+        <v>27.051806636487068</v>
+      </c>
+      <c r="E48" s="5">
+        <f>_xlfn.STDEV.S(E2:E46)</f>
+        <v>11.959662616068906</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>8</v>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5">
+        <f>_xlfn.STDEV.S(C2:C46)/SQRT(COUNT(C2:C46))</f>
+        <v>2.31056141495311</v>
+      </c>
+      <c r="D49" s="5">
+        <f>_xlfn.STDEV.S(D2:D46)/SQRT(COUNT(D2:D46))</f>
+        <v>4.0326452368910015</v>
+      </c>
+      <c r="E49" s="5">
+        <f>E48/SQRT(COUNT(E2:E46))</f>
+        <v>1.7828412398328695</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5">
+        <f>C47/C49</f>
+        <v>24.611166343985559</v>
+      </c>
+      <c r="D50" s="5">
+        <f>D47/D49</f>
+        <v>20.891953242652804</v>
+      </c>
+      <c r="E50" s="5">
+        <f>E47/E49</f>
+        <v>15.359878260666003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5">
+        <f>2*_xlfn.T.DIST.2T(ABS(C50), COUNT(C2:C46)-1)</f>
+        <v>4.6715012553319779E-27</v>
+      </c>
+      <c r="D51" s="5">
+        <f>2*_xlfn.T.DIST.2T(ABS(D50), COUNT(D2:D46)-1)</f>
+        <v>3.6133689414669986E-24</v>
+      </c>
+      <c r="E51" s="6">
+        <f>2*_xlfn.T.DIST.2T(ABS(E50), COUNT(E2:E46)-1)</f>
+        <v>5.4347350488387664E-19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>